<commit_message>
Update template export doc control for row border auto increament
</commit_message>
<xml_diff>
--- a/public/template_excel/Document-Control.xlsx
+++ b/public/template_excel/Document-Control.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Syifa\donnav2\public\template_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{612235E6-438D-452C-B7A5-5AE5951E6563}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36C76FDB-9C3E-494E-B54C-51128BA0CA15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{2043A8B8-C64B-45E1-B5AE-CF5A4A4F0B09}"/>
   </bookViews>
@@ -184,28 +184,28 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -578,67 +578,67 @@
       <c r="F2" s="4"/>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="9"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="8"/>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="8"/>
+      <c r="C6" s="6"/>
       <c r="D6" s="1"/>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="C7" s="8"/>
+      <c r="C7" s="6"/>
       <c r="D7" s="1"/>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="8"/>
+      <c r="C8" s="6"/>
       <c r="D8" s="1"/>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="F10" s="9" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="6"/>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="10"/>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B12" s="1"/>

</xml_diff>

<commit_message>
Update excvel template doc control use filter
</commit_message>
<xml_diff>
--- a/public/template_excel/Document-Control.xlsx
+++ b/public/template_excel/Document-Control.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Syifa\donnav2\public\template_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36C76FDB-9C3E-494E-B54C-51128BA0CA15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C274585-EA5F-4DC8-8CC1-A4D27892A481}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{2043A8B8-C64B-45E1-B5AE-CF5A4A4F0B09}"/>
   </bookViews>
   <sheets>
     <sheet name="Document Control" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Document Control'!$C$10:$F$11</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -3812,6 +3815,7 @@
       <c r="F464" s="1"/>
     </row>
   </sheetData>
+  <autoFilter ref="C10:F11" xr:uid="{8CA131CD-9906-42CC-A00B-BCCB48CD3738}"/>
   <mergeCells count="12">
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B2:F2"/>

</xml_diff>